<commit_message>
docs(week5): rewrite day-1-2 ticket analysis report for login automation
</commit_message>
<xml_diff>
--- a/week-5/odoo-automation/week-5/Phiếu hỗ trợ (helpdesk.ticket).xlsx
+++ b/week-5/odoo-automation/week-5/Phiếu hỗ trợ (helpdesk.ticket).xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="98">
   <si>
     <t>Đang hoạt động</t>
   </si>
@@ -94,7 +94,7 @@
     <t>Thuộc tính 1</t>
   </si>
   <si>
-    <t>Mới (4)</t>
+    <t>Mới (3)</t>
   </si>
   <si>
     <t>0</t>
@@ -103,73 +103,85 @@
     <t>Chăm sóc khách hàng</t>
   </si>
   <si>
+    <t>ko login dc - Tran Thi B</t>
+  </si>
+  <si>
+    <t>00019</t>
+  </si>
+  <si>
+    <t>Trần Thị B</t>
+  </si>
+  <si>
+    <t>Ưu tiên trung bình</t>
+  </si>
+  <si>
+    <t>Anh Mỹ</t>
+  </si>
+  <si>
+    <t>Đang thực hiện</t>
+  </si>
+  <si>
+    <t>Không tải được tài liệu bài 5 - HV Lê Thị E</t>
+  </si>
+  <si>
+    <t>00013</t>
+  </si>
+  <si>
+    <t>Lê Thị E</t>
+  </si>
+  <si>
+    <t>LMS</t>
+  </si>
+  <si>
+    <t>content</t>
+  </si>
+  <si>
+    <t>LMS login failed - Teacher Phạm Văn C</t>
+  </si>
+  <si>
+    <t>00012</t>
+  </si>
+  <si>
+    <t>Phạm Văn C</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>teacher</t>
+  </si>
+  <si>
+    <t>Đang thực hiện (6)</t>
+  </si>
+  <si>
+    <t>không đăng nhập được - anhmy</t>
+  </si>
+  <si>
+    <t>00023</t>
+  </si>
+  <si>
+    <t>Anh My</t>
+  </si>
+  <si>
+    <t>Login hỏng</t>
+  </si>
+  <si>
+    <t>00022</t>
+  </si>
+  <si>
+    <t>anhmy1</t>
+  </si>
+  <si>
+    <t>login lỗi</t>
+  </si>
+  <si>
+    <t>00021</t>
+  </si>
+  <si>
     <t>login lỗi - anh my</t>
   </si>
   <si>
     <t>00020</t>
-  </si>
-  <si>
-    <t>Anh My</t>
-  </si>
-  <si>
-    <t>LMS</t>
-  </si>
-  <si>
-    <t>Ưu tiên trung bình</t>
-  </si>
-  <si>
-    <t>Anh Mỹ</t>
-  </si>
-  <si>
-    <t>Đang thực hiện</t>
-  </si>
-  <si>
-    <t>Login</t>
-  </si>
-  <si>
-    <t>ko login dc - Tran Thi B</t>
-  </si>
-  <si>
-    <t>00019</t>
-  </si>
-  <si>
-    <t>Trần Thị B</t>
-  </si>
-  <si>
-    <t>Không tải được tài liệu bài 5 - HV Lê Thị E</t>
-  </si>
-  <si>
-    <t>00013</t>
-  </si>
-  <si>
-    <t>Lê Thị E</t>
-  </si>
-  <si>
-    <t>content</t>
-  </si>
-  <si>
-    <t>LMS login failed - Teacher Phạm Văn C</t>
-  </si>
-  <si>
-    <t>00012</t>
-  </si>
-  <si>
-    <t>Phạm Văn C</t>
-  </si>
-  <si>
-    <t>teacher</t>
-  </si>
-  <si>
-    <t>Đang thực hiện (3)</t>
-  </si>
-  <si>
-    <t>login lỗi</t>
-  </si>
-  <si>
-    <t>00021</t>
-  </si>
-  <si>
-    <t>anhmy1</t>
   </si>
   <si>
     <t>Login - Nguyễn Thị D</t>
@@ -657,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z43"/>
+  <dimension ref="A1:Z46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="26" width="30.7109375" customWidth="1"/>
@@ -817,24 +829,22 @@
       <c r="M3" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="N3" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" s="4">
+        <v>0</v>
+      </c>
+      <c r="S3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Q3" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4">
-        <v>0</v>
-      </c>
-      <c r="S3" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
@@ -844,28 +854,60 @@
       <c r="Z3" s="4"/>
     </row>
     <row r="4" spans="1:26">
-      <c r="A4" s="4"/>
+      <c r="A4" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="N4" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
+      <c r="P4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" s="4">
+        <v>0</v>
+      </c>
+      <c r="S4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U4" s="4"/>
       <c r="V4" s="4"/>
       <c r="W4" s="4"/>
@@ -874,58 +916,28 @@
       <c r="Z4" s="4"/>
     </row>
     <row r="5" spans="1:26">
-      <c r="A5" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I5" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" s="4">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="M5" s="4" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="N5" s="4"/>
       <c r="O5" s="4"/>
-      <c r="P5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R5" s="4">
-        <v>0</v>
-      </c>
-      <c r="S5" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T5" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -970,23 +982,23 @@
         <v>42</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="O6" s="4"/>
       <c r="P6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" s="4">
+        <v>0</v>
+      </c>
+      <c r="S6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Q6" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R6" s="4">
-        <v>0</v>
-      </c>
-      <c r="S6" s="4" t="s">
+      <c r="T6" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="T6" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="U6" s="4"/>
       <c r="V6" s="4"/>
@@ -1026,60 +1038,28 @@
       <c r="Z7" s="4"/>
     </row>
     <row r="8" spans="1:26">
-      <c r="A8" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" s="4">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="L8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="O8" s="4"/>
-      <c r="P8" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R8" s="4">
-        <v>0</v>
-      </c>
-      <c r="S8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T8" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
@@ -1088,58 +1068,96 @@
       <c r="Z8" s="4"/>
     </row>
     <row r="9" spans="1:26">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="4"/>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="4"/>
+      <c r="A9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
+      <c r="X9" s="2"/>
+      <c r="Y9" s="2"/>
+      <c r="Z9" s="2"/>
     </row>
     <row r="10" spans="1:26">
-      <c r="A10" s="4"/>
+      <c r="A10" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4" t="s">
+      <c r="D10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="4">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L10" s="4" t="s">
         <v>47</v>
       </c>
+      <c r="M10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N10" s="4"/>
       <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
+      <c r="P10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q10" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T10" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U10" s="4"/>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
@@ -1148,98 +1166,90 @@
       <c r="Z10" s="4"/>
     </row>
     <row r="11" spans="1:26">
-      <c r="A11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="3">
-        <v>0</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-      <c r="Y11" s="2"/>
-      <c r="Z11" s="2"/>
+      <c r="A11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" s="4">
+        <v>0</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
+      <c r="W11" s="4"/>
+      <c r="X11" s="4"/>
+      <c r="Y11" s="4"/>
+      <c r="Z11" s="4"/>
     </row>
     <row r="12" spans="1:26">
-      <c r="A12" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
-      <c r="D12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I12" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J12" s="4">
-        <v>0</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>51</v>
-      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
       <c r="N12" s="4" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="O12" s="4"/>
-      <c r="P12" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q12" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R12" s="4">
-        <v>0</v>
-      </c>
-      <c r="S12" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T12" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
       <c r="U12" s="4"/>
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
@@ -1248,28 +1258,60 @@
       <c r="Z12" s="4"/>
     </row>
     <row r="13" spans="1:26">
-      <c r="A13" s="4"/>
+      <c r="A13" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
+      <c r="D13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>51</v>
+      </c>
       <c r="N13" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O13" s="4"/>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="4"/>
-      <c r="S13" s="4"/>
-      <c r="T13" s="4"/>
+      <c r="P13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q13" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" s="4">
+        <v>0</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U13" s="4"/>
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
@@ -1278,60 +1320,28 @@
       <c r="Z13" s="4"/>
     </row>
     <row r="14" spans="1:26">
-      <c r="A14" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F14" s="4">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I14" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J14" s="4">
-        <v>0</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>54</v>
-      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
       <c r="N14" s="4" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="O14" s="4"/>
-      <c r="P14" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q14" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R14" s="4">
-        <v>0</v>
-      </c>
-      <c r="S14" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T14" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4"/>
+      <c r="R14" s="4"/>
+      <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
       <c r="U14" s="4"/>
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
@@ -1340,28 +1350,60 @@
       <c r="Z14" s="4"/>
     </row>
     <row r="15" spans="1:26">
-      <c r="A15" s="4"/>
+      <c r="A15" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
+      <c r="D15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" s="4">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>48</v>
+      </c>
       <c r="N15" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O15" s="4"/>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
+      <c r="P15" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q15" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R15" s="4">
+        <v>0</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T15" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U15" s="4"/>
       <c r="V15" s="4"/>
       <c r="W15" s="4"/>
@@ -1370,60 +1412,28 @@
       <c r="Z15" s="4"/>
     </row>
     <row r="16" spans="1:26">
-      <c r="A16" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F16" s="4">
-        <v>0</v>
-      </c>
-      <c r="G16" s="5">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I16" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J16" s="4">
-        <v>0</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="L16" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>39</v>
-      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
       <c r="N16" s="4" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="O16" s="4"/>
-      <c r="P16" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q16" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R16" s="4">
-        <v>0</v>
-      </c>
-      <c r="S16" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T16" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+      <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
       <c r="U16" s="4"/>
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
@@ -1432,28 +1442,60 @@
       <c r="Z16" s="4"/>
     </row>
     <row r="17" spans="1:26">
-      <c r="A17" s="4"/>
+      <c r="A17" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
+      <c r="D17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" s="4">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>58</v>
+      </c>
       <c r="N17" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O17" s="4"/>
-      <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
-      <c r="S17" s="4"/>
-      <c r="T17" s="4"/>
+      <c r="P17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q17" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R17" s="4">
+        <v>0</v>
+      </c>
+      <c r="S17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T17" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U17" s="4"/>
       <c r="V17" s="4"/>
       <c r="W17" s="4"/>
@@ -1476,7 +1518,7 @@
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
@@ -1492,98 +1534,90 @@
       <c r="Z18" s="4"/>
     </row>
     <row r="19" spans="1:26">
-      <c r="A19" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G19" s="3">
-        <v>0</v>
-      </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
-      <c r="X19" s="2"/>
-      <c r="Y19" s="2"/>
-      <c r="Z19" s="2"/>
+      <c r="A19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" s="4">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q19" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19" s="4">
+        <v>0</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T19" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
+      <c r="W19" s="4"/>
+      <c r="X19" s="4"/>
+      <c r="Y19" s="4"/>
+      <c r="Z19" s="4"/>
     </row>
     <row r="20" spans="1:26">
-      <c r="A20" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A20" s="4"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F20" s="4">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5">
-        <v>0</v>
-      </c>
-      <c r="H20" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J20" s="4">
-        <v>0</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="L20" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>60</v>
-      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
       <c r="N20" s="4" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="O20" s="4"/>
-      <c r="P20" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q20" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R20" s="4">
-        <v>0</v>
-      </c>
-      <c r="S20" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T20" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
       <c r="U20" s="4"/>
       <c r="V20" s="4"/>
       <c r="W20" s="4"/>
@@ -1606,7 +1640,7 @@
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
       <c r="N21" s="4" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="O21" s="4"/>
       <c r="P21" s="4"/>
@@ -1622,58 +1656,98 @@
       <c r="Z21" s="4"/>
     </row>
     <row r="22" spans="1:26">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
-      <c r="V22" s="4"/>
-      <c r="W22" s="4"/>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="4"/>
-      <c r="Z22" s="4"/>
+      <c r="A22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="3">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22" s="2"/>
+      <c r="V22" s="2"/>
+      <c r="W22" s="2"/>
+      <c r="X22" s="2"/>
+      <c r="Y22" s="2"/>
+      <c r="Z22" s="2"/>
     </row>
     <row r="23" spans="1:26">
-      <c r="A23" s="4"/>
+      <c r="A23" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
+      <c r="D23" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J23" s="4">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>64</v>
+      </c>
       <c r="N23" s="4" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="O23" s="4"/>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="4"/>
-      <c r="S23" s="4"/>
-      <c r="T23" s="4"/>
+      <c r="P23" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q23" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R23" s="4">
+        <v>0</v>
+      </c>
+      <c r="S23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T23" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
       <c r="W23" s="4"/>
@@ -1682,60 +1756,28 @@
       <c r="Z23" s="4"/>
     </row>
     <row r="24" spans="1:26">
-      <c r="A24" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A24" s="4"/>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E24" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F24" s="4">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5">
-        <v>0</v>
-      </c>
-      <c r="H24" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I24" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J24" s="4">
-        <v>0</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="L24" s="4" t="s">
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="M24" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="N24" s="4" t="s">
-        <v>68</v>
-      </c>
       <c r="O24" s="4"/>
-      <c r="P24" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q24" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R24" s="4">
-        <v>0</v>
-      </c>
-      <c r="S24" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T24" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
       <c r="U24" s="4"/>
       <c r="V24" s="4"/>
       <c r="W24" s="4"/>
@@ -1758,7 +1800,7 @@
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
       <c r="N25" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
@@ -1788,7 +1830,7 @@
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
       <c r="N26" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
@@ -1804,28 +1846,60 @@
       <c r="Z26" s="4"/>
     </row>
     <row r="27" spans="1:26">
-      <c r="A27" s="4"/>
+      <c r="A27" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
+      <c r="D27" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E27" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J27" s="4">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>71</v>
+      </c>
       <c r="N27" s="4" t="s">
         <v>72</v>
       </c>
       <c r="O27" s="4"/>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-      <c r="R27" s="4"/>
-      <c r="S27" s="4"/>
-      <c r="T27" s="4"/>
+      <c r="P27" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q27" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27" s="4">
+        <v>0</v>
+      </c>
+      <c r="S27" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T27" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U27" s="4"/>
       <c r="V27" s="4"/>
       <c r="W27" s="4"/>
@@ -1834,58 +1908,28 @@
       <c r="Z27" s="4"/>
     </row>
     <row r="28" spans="1:26">
-      <c r="A28" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
-      <c r="D28" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F28" s="4">
-        <v>0</v>
-      </c>
-      <c r="G28" s="5">
-        <v>0</v>
-      </c>
-      <c r="H28" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I28" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J28" s="4">
-        <v>0</v>
-      </c>
-      <c r="K28" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="L28" s="4" t="s">
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="M28" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="N28" s="4"/>
       <c r="O28" s="4"/>
-      <c r="P28" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q28" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R28" s="4">
-        <v>0</v>
-      </c>
-      <c r="S28" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T28" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
+      <c r="R28" s="4"/>
+      <c r="S28" s="4"/>
+      <c r="T28" s="4"/>
       <c r="U28" s="4"/>
       <c r="V28" s="4"/>
       <c r="W28" s="4"/>
@@ -1894,58 +1938,28 @@
       <c r="Z28" s="4"/>
     </row>
     <row r="29" spans="1:26">
-      <c r="A29" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
-      <c r="D29" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E29" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F29" s="4">
-        <v>0</v>
-      </c>
-      <c r="G29" s="5">
-        <v>0</v>
-      </c>
-      <c r="H29" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J29" s="4">
-        <v>0</v>
-      </c>
-      <c r="K29" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="L29" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="M29" s="4" t="s">
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="N29" s="4"/>
       <c r="O29" s="4"/>
-      <c r="P29" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q29" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R29" s="4">
-        <v>0</v>
-      </c>
-      <c r="S29" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T29" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
+      <c r="R29" s="4"/>
+      <c r="S29" s="4"/>
+      <c r="T29" s="4"/>
       <c r="U29" s="4"/>
       <c r="V29" s="4"/>
       <c r="W29" s="4"/>
@@ -1954,58 +1968,28 @@
       <c r="Z29" s="4"/>
     </row>
     <row r="30" spans="1:26">
-      <c r="A30" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
-      <c r="D30" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E30" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F30" s="4">
-        <v>0</v>
-      </c>
-      <c r="G30" s="5">
-        <v>0</v>
-      </c>
-      <c r="H30" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I30" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J30" s="4">
-        <v>0</v>
-      </c>
-      <c r="K30" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="L30" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="M30" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="N30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4" t="s">
+        <v>76</v>
+      </c>
       <c r="O30" s="4"/>
-      <c r="P30" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q30" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R30" s="4">
-        <v>0</v>
-      </c>
-      <c r="S30" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T30" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P30" s="4"/>
+      <c r="Q30" s="4"/>
+      <c r="R30" s="4"/>
+      <c r="S30" s="4"/>
+      <c r="T30" s="4"/>
       <c r="U30" s="4"/>
       <c r="V30" s="4"/>
       <c r="W30" s="4"/>
@@ -2041,20 +2025,18 @@
         <v>0</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="L31" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="M31" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="N31" s="4" t="s">
-        <v>32</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="N31" s="4"/>
       <c r="O31" s="4"/>
       <c r="P31" s="4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="Q31" s="4" t="b">
         <v>0</v>
@@ -2063,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="S31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T31" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="T31" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="U31" s="4"/>
       <c r="V31" s="4"/>
@@ -2076,28 +2058,58 @@
       <c r="Z31" s="4"/>
     </row>
     <row r="32" spans="1:26">
-      <c r="A32" s="4"/>
+      <c r="A32" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4" t="s">
-        <v>83</v>
-      </c>
+      <c r="D32" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5">
+        <v>0</v>
+      </c>
+      <c r="H32" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" s="4">
+        <v>0</v>
+      </c>
+      <c r="K32" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="N32" s="4"/>
       <c r="O32" s="4"/>
-      <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-      <c r="R32" s="4"/>
-      <c r="S32" s="4"/>
-      <c r="T32" s="4"/>
+      <c r="P32" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q32" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R32" s="4">
+        <v>0</v>
+      </c>
+      <c r="S32" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T32" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U32" s="4"/>
       <c r="V32" s="4"/>
       <c r="W32" s="4"/>
@@ -2106,28 +2118,58 @@
       <c r="Z32" s="4"/>
     </row>
     <row r="33" spans="1:26">
-      <c r="A33" s="4"/>
+      <c r="A33" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4" t="s">
-        <v>84</v>
-      </c>
+      <c r="D33" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E33" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F33" s="4">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" s="4">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="L33" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="M33" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="N33" s="4"/>
       <c r="O33" s="4"/>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-      <c r="S33" s="4"/>
-      <c r="T33" s="4"/>
+      <c r="P33" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q33" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R33" s="4">
+        <v>0</v>
+      </c>
+      <c r="S33" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T33" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U33" s="4"/>
       <c r="V33" s="4"/>
       <c r="W33" s="4"/>
@@ -2136,28 +2178,60 @@
       <c r="Z33" s="4"/>
     </row>
     <row r="34" spans="1:26">
-      <c r="A34" s="4"/>
+      <c r="A34" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
+      <c r="D34" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34" s="4">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I34" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J34" s="4">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>86</v>
+      </c>
       <c r="N34" s="4" t="s">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="O34" s="4"/>
-      <c r="P34" s="4"/>
-      <c r="Q34" s="4"/>
-      <c r="R34" s="4"/>
-      <c r="S34" s="4"/>
-      <c r="T34" s="4"/>
+      <c r="P34" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q34" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R34" s="4">
+        <v>0</v>
+      </c>
+      <c r="S34" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T34" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="U34" s="4"/>
       <c r="V34" s="4"/>
       <c r="W34" s="4"/>
@@ -2166,60 +2240,28 @@
       <c r="Z34" s="4"/>
     </row>
     <row r="35" spans="1:26">
-      <c r="A35" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
-      <c r="D35" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E35" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F35" s="4">
-        <v>0</v>
-      </c>
-      <c r="G35" s="5">
-        <v>0</v>
-      </c>
-      <c r="H35" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I35" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J35" s="4">
-        <v>0</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="L35" s="4" t="s">
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="M35" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="N35" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="O35" s="4"/>
-      <c r="P35" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q35" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R35" s="4">
-        <v>0</v>
-      </c>
-      <c r="S35" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="T35" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="P35" s="4"/>
+      <c r="Q35" s="4"/>
+      <c r="R35" s="4"/>
+      <c r="S35" s="4"/>
+      <c r="T35" s="4"/>
       <c r="U35" s="4"/>
       <c r="V35" s="4"/>
       <c r="W35" s="4"/>
@@ -2242,7 +2284,7 @@
       <c r="L36" s="4"/>
       <c r="M36" s="4"/>
       <c r="N36" s="4" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="O36" s="4"/>
       <c r="P36" s="4"/>
@@ -2272,7 +2314,7 @@
       <c r="L37" s="4"/>
       <c r="M37" s="4"/>
       <c r="N37" s="4" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="O37" s="4"/>
       <c r="P37" s="4"/>
@@ -2315,32 +2357,32 @@
         <v>0</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L38" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="M38" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N38" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="O38" s="4"/>
       <c r="P38" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q38" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R38" s="4">
+        <v>0</v>
+      </c>
+      <c r="S38" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Q38" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R38" s="4">
-        <v>0</v>
-      </c>
-      <c r="S38" s="4" t="s">
+      <c r="T38" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="T38" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="U38" s="4"/>
       <c r="V38" s="4"/>
@@ -2364,7 +2406,7 @@
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
       <c r="N39" s="4" t="s">
-        <v>92</v>
+        <v>43</v>
       </c>
       <c r="O39" s="4"/>
       <c r="P39" s="4"/>
@@ -2394,7 +2436,7 @@
       <c r="L40" s="4"/>
       <c r="M40" s="4"/>
       <c r="N40" s="4" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="O40" s="4"/>
       <c r="P40" s="4"/>
@@ -2437,32 +2479,32 @@
         <v>0</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="L41" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M41" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="N41" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="O41" s="4"/>
       <c r="P41" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q41" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R41" s="4">
+        <v>0</v>
+      </c>
+      <c r="S41" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Q41" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R41" s="4">
-        <v>0</v>
-      </c>
-      <c r="S41" s="4" t="s">
+      <c r="T41" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="T41" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="U41" s="4"/>
       <c r="V41" s="4"/>
@@ -2486,7 +2528,7 @@
       <c r="L42" s="4"/>
       <c r="M42" s="4"/>
       <c r="N42" s="4" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="O42" s="4"/>
       <c r="P42" s="4"/>
@@ -2516,7 +2558,7 @@
       <c r="L43" s="4"/>
       <c r="M43" s="4"/>
       <c r="N43" s="4" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="O43" s="4"/>
       <c r="P43" s="4"/>
@@ -2531,6 +2573,128 @@
       <c r="Y43" s="4"/>
       <c r="Z43" s="4"/>
     </row>
+    <row r="44" spans="1:26">
+      <c r="A44" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E44" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F44" s="4">
+        <v>0</v>
+      </c>
+      <c r="G44" s="5">
+        <v>0</v>
+      </c>
+      <c r="H44" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I44" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J44" s="4">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="L44" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="M44" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="N44" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O44" s="4"/>
+      <c r="P44" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q44" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R44" s="4">
+        <v>0</v>
+      </c>
+      <c r="S44" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T44" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="U44" s="4"/>
+      <c r="V44" s="4"/>
+      <c r="W44" s="4"/>
+      <c r="X44" s="4"/>
+      <c r="Y44" s="4"/>
+      <c r="Z44" s="4"/>
+    </row>
+    <row r="45" spans="1:26">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+      <c r="N45" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="O45" s="4"/>
+      <c r="P45" s="4"/>
+      <c r="Q45" s="4"/>
+      <c r="R45" s="4"/>
+      <c r="S45" s="4"/>
+      <c r="T45" s="4"/>
+      <c r="U45" s="4"/>
+      <c r="V45" s="4"/>
+      <c r="W45" s="4"/>
+      <c r="X45" s="4"/>
+      <c r="Y45" s="4"/>
+      <c r="Z45" s="4"/>
+    </row>
+    <row r="46" spans="1:26">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="4"/>
+      <c r="T46" s="4"/>
+      <c r="U46" s="4"/>
+      <c r="V46" s="4"/>
+      <c r="W46" s="4"/>
+      <c r="X46" s="4"/>
+      <c r="Y46" s="4"/>
+      <c r="Z46" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>